<commit_message>
Updated VNM model - 2025-12-12 15:35
</commit_message>
<xml_diff>
--- a/VerveStacks_VNM/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_VNM/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_VNM\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7B496D26-E4EC-4FFA-99FD-21BC4EE0ECA9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{18B76B50-0176-4D24-AF1D-BB35E90ABA50}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="6" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -56,7 +56,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1292" uniqueCount="392">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1293" uniqueCount="394">
   <si>
     <t>~FI_Process</t>
   </si>
@@ -618,6 +618,9 @@
     <t>wnid offshore potential</t>
   </si>
   <si>
+    <t>ELC_BatIn</t>
+  </si>
+  <si>
     <t>~fi_process</t>
   </si>
   <si>
@@ -1303,6 +1306,9 @@
   </si>
   <si>
     <t>yes</t>
+  </si>
+  <si>
+    <t>e_VN1003-500,e_VN1005-500,e_VN1008-500,e_VN1010-500,e_VN1014-500,e_VN1016-500,e_VN1019-500,e_VN1020-500,e_VN1022-500,e_VN1024-220,e_VN1130-500,e_VN1133-220,e_VN1134-220,e_VN1137-500,e_VN1138-220,e_VN1139-220,e_VN1140-500,e_VN1141-220,e_VN1141-500,e_VN1142-500,e_VN1145-220,e_VN1146-500,e_VN1147-220,e_VN1149-500,e_VN1153-220,e_VN1154-220,e_VN1157-220,e_VN1178-500,e_VN1179-220,e_VN1184-500,e_VN1187-500,e_VN1188-220,e_VN1191-500,e_VN1192-500,e_VN1196-500,e_VN1198-500,e_VN1206-220,e_VN1208-500,e_VN1209-500,e_VN1210-500,e_VN1213-220,e_VN1218-220,e_VN1219-220,e_VN1223-220,e_VN1223-500,e_VN1224-500,e_VN1226-500,e_VN1228-220,e_VN181-500,e_VN183-500,e_VN186-500,e_VN188-500,e_VN189-500,e_VN192-500,e_VN195-220,e_VN195-500,e_VN196-500,e_VN197-500,e_VN198-500,e_VN199-500,e_VN2-220,e_VN200-500,e_VN201-500,e_VN202-500,e_VN203-220,e_VN203-500,e_VN205-500,e_VN206-500,e_VN207-500,e_VN209-220,e_VN210-500,e_VN211-500,e_VN212-500,e_VN213-500,e_VN214-500,e_VN215-500,e_VN216-500,e_VN217-500,e_VN218-500,e_VN224-500,e_VN225-500,e_VN226-500,e_VN229-500,e_VN230-220,e_VN230-500,e_VN232-220,e_VN251-220,e_VN252-220,e_VN274-220,e_VN310-220,e_VN323-500,e_VN328-500,e_VN334-500,e_VN365-220,e_VN383-220,e_VN391-500,e_VN392-500,e_VN393-500,e_VN394-500,e_VN395-500,e_VN396-500,e_VN397-500,e_VN398-500,e_VN400-500,e_VN401-500,e_VN402-500,e_VN404-500,e_VN405-500,e_VN406-500,e_VN408-220,e_VN408-500,e_VN409-500,e_VN410-220,e_VN411-500,e_VN412-500,e_VN413-220,e_VN414-500,e_VN418-500,e_VN419-500,e_VN421-500,e_VN422-500,e_VN427-500,e_VN428-500,e_VN429-500,e_VN430-500,e_VN431-500,e_VN432-500,e_VN433-500,e_VN434-500,e_VN435-500,e_VN436-500,e_VN437-500,e_VN438-500,e_VN439-500,e_VN440-500,e_VN441-500,e_VN442-500,e_VN449-500,e_VN451-220,e_VN452-500,e_VN454-500,e_VN455-500,e_VN509-500,e_VN511-220,e_VN511-500,e_VN512-500,e_VN513-500,e_VN514-500,e_VN515-500,e_VN516-500,e_VN517-500,e_VN518-500,e_VN519-220,e_VN519-500,e_VN520-500,e_VN521-220,e_VN521-500,e_VN522-500,e_VN523-500,e_VN524-500,e_VN525-500,e_VN526-500,e_VN527-500,e_VN528-500,e_VN529-500,e_VN533-220,e_VN534-220,e_VN534-500,e_VN536-220,e_VN537-220,e_VN538-220,e_VN539-220,e_VN540-220,e_VN589-500,e_VN592-500,e_VN595-500,e_VN597-500,e_VN598-500,e_VN624-220,e_VN801-500,e_VN802-500,e_VN803-500,e_VN805-500,e_VN806-500,e_VN807-500,e_VN813-500,e_VN814-500,e_VN815-500,e_VN819-500,e_VN823-500,e_VN824-500,e_VN825-500,e_VN826-500,e_VN836-220,e_VN837-220,e_VN902-220,e_VN937-220,e_VN988-220,e_VN994-500,e_VN998-500,e_VN999-500,e_w1018528434-220,e_w1044469623-220,e_w1045125739-220,e_w1047280375-220,e_w1047400696-220,e_w1047400696-500,e_w1052065872-220,e_w1052125064-220,e_w1087113517-220,e_w1091686589-220,e_w1091782693-220,e_w1176845159-220,e_w1176845164-220,e_w1183902227-500,e_w1216970886-220,e_w1216970886-500,e_w1245195233-220,e_w1258175914-220,e_w1265274413-220,e_w1265274426-500,e_w1265612937-220,e_w1272088369-220,e_w1273255946-220,e_w1273527149-220,e_w1273527210-220,e_w1273948701-220,e_w1274076450-220,e_w1274076450-500,e_w1274466549-220,e_w1320784083-220,e_w1320784083-500,e_w1374565925-220,e_w1376430795-220,e_w1376430795-500,e_w241065371-220,e_w306295536-220,e_w306295536-500,e_w306295540-220,e_w307638314-220,e_w315766007-220,e_w315766015-220,e_w400645442-220,e_w400791086-220,e_w400791086-500,e_w401042494-220,e_w401532710-220,e_w468821783-220,e_w468821783-500,e_w548717060-220,e_w548717060-500,e_w548723124-220,e_w548752026-220,e_w548869165-220,e_w548869165-230,e_w548970118-220,e_w549038673-220,e_w549296358-220,e_w549380074-220,e_w549400050-220,e_w549400050-500,e_w549400051-220,e_w549577079-220,e_w549914200-220,e_w549941525-220,e_w549959350-220,e_w549959354-220,e_w630750798-220,e_w630750798-500,e_w715041211-220,e_w744217936-220,e_w762471641-220,e_w827889590-500,e_w827889600-220,e_w827889600-500,e_w967849373-220</t>
   </si>
 </sst>
 </file>
@@ -3196,7 +3202,7 @@
       </c>
       <c r="L27" t="str">
         <f>$V$28</f>
-        <v>ELC</v>
+        <v>e_VN1003-500,e_VN1005-500,e_VN1008-500,e_VN1010-500,e_VN1014-500,e_VN1016-500,e_VN1019-500,e_VN1020-500,e_VN1022-500,e_VN1024-220,e_VN1130-500,e_VN1133-220,e_VN1134-220,e_VN1137-500,e_VN1138-220,e_VN1139-220,e_VN1140-500,e_VN1141-220,e_VN1141-500,e_VN1142-500,e_VN1145-220,e_VN1146-500,e_VN1147-220,e_VN1149-500,e_VN1153-220,e_VN1154-220,e_VN1157-220,e_VN1178-500,e_VN1179-220,e_VN1184-500,e_VN1187-500,e_VN1188-220,e_VN1191-500,e_VN1192-500,e_VN1196-500,e_VN1198-500,e_VN1206-220,e_VN1208-500,e_VN1209-500,e_VN1210-500,e_VN1213-220,e_VN1218-220,e_VN1219-220,e_VN1223-220,e_VN1223-500,e_VN1224-500,e_VN1226-500,e_VN1228-220,e_VN181-500,e_VN183-500,e_VN186-500,e_VN188-500,e_VN189-500,e_VN192-500,e_VN195-220,e_VN195-500,e_VN196-500,e_VN197-500,e_VN198-500,e_VN199-500,e_VN2-220,e_VN200-500,e_VN201-500,e_VN202-500,e_VN203-220,e_VN203-500,e_VN205-500,e_VN206-500,e_VN207-500,e_VN209-220,e_VN210-500,e_VN211-500,e_VN212-500,e_VN213-500,e_VN214-500,e_VN215-500,e_VN216-500,e_VN217-500,e_VN218-500,e_VN224-500,e_VN225-500,e_VN226-500,e_VN229-500,e_VN230-220,e_VN230-500,e_VN232-220,e_VN251-220,e_VN252-220,e_VN274-220,e_VN310-220,e_VN323-500,e_VN328-500,e_VN334-500,e_VN365-220,e_VN383-220,e_VN391-500,e_VN392-500,e_VN393-500,e_VN394-500,e_VN395-500,e_VN396-500,e_VN397-500,e_VN398-500,e_VN400-500,e_VN401-500,e_VN402-500,e_VN404-500,e_VN405-500,e_VN406-500,e_VN408-220,e_VN408-500,e_VN409-500,e_VN410-220,e_VN411-500,e_VN412-500,e_VN413-220,e_VN414-500,e_VN418-500,e_VN419-500,e_VN421-500,e_VN422-500,e_VN427-500,e_VN428-500,e_VN429-500,e_VN430-500,e_VN431-500,e_VN432-500,e_VN433-500,e_VN434-500,e_VN435-500,e_VN436-500,e_VN437-500,e_VN438-500,e_VN439-500,e_VN440-500,e_VN441-500,e_VN442-500,e_VN449-500,e_VN451-220,e_VN452-500,e_VN454-500,e_VN455-500,e_VN509-500,e_VN511-220,e_VN511-500,e_VN512-500,e_VN513-500,e_VN514-500,e_VN515-500,e_VN516-500,e_VN517-500,e_VN518-500,e_VN519-220,e_VN519-500,e_VN520-500,e_VN521-220,e_VN521-500,e_VN522-500,e_VN523-500,e_VN524-500,e_VN525-500,e_VN526-500,e_VN527-500,e_VN528-500,e_VN529-500,e_VN533-220,e_VN534-220,e_VN534-500,e_VN536-220,e_VN537-220,e_VN538-220,e_VN539-220,e_VN540-220,e_VN589-500,e_VN592-500,e_VN595-500,e_VN597-500,e_VN598-500,e_VN624-220,e_VN801-500,e_VN802-500,e_VN803-500,e_VN805-500,e_VN806-500,e_VN807-500,e_VN813-500,e_VN814-500,e_VN815-500,e_VN819-500,e_VN823-500,e_VN824-500,e_VN825-500,e_VN826-500,e_VN836-220,e_VN837-220,e_VN902-220,e_VN937-220,e_VN988-220,e_VN994-500,e_VN998-500,e_VN999-500,e_w1018528434-220,e_w1044469623-220,e_w1045125739-220,e_w1047280375-220,e_w1047400696-220,e_w1047400696-500,e_w1052065872-220,e_w1052125064-220,e_w1087113517-220,e_w1091686589-220,e_w1091782693-220,e_w1176845159-220,e_w1176845164-220,e_w1183902227-500,e_w1216970886-220,e_w1216970886-500,e_w1245195233-220,e_w1258175914-220,e_w1265274413-220,e_w1265274426-500,e_w1265612937-220,e_w1272088369-220,e_w1273255946-220,e_w1273527149-220,e_w1273527210-220,e_w1273948701-220,e_w1274076450-220,e_w1274076450-500,e_w1274466549-220,e_w1320784083-220,e_w1320784083-500,e_w1374565925-220,e_w1376430795-220,e_w1376430795-500,e_w241065371-220,e_w306295536-220,e_w306295536-500,e_w306295540-220,e_w307638314-220,e_w315766007-220,e_w315766015-220,e_w400645442-220,e_w400791086-220,e_w400791086-500,e_w401042494-220,e_w401532710-220,e_w468821783-220,e_w468821783-500,e_w548717060-220,e_w548717060-500,e_w548723124-220,e_w548752026-220,e_w548869165-220,e_w548869165-230,e_w548970118-220,e_w549038673-220,e_w549296358-220,e_w549380074-220,e_w549400050-220,e_w549400050-500,e_w549400051-220,e_w549577079-220,e_w549914200-220,e_w549941525-220,e_w549959350-220,e_w549959354-220,e_w630750798-220,e_w630750798-500,e_w715041211-220,e_w744217936-220,e_w762471641-220,e_w827889590-500,e_w827889600-220,e_w827889600-500,e_w967849373-220</v>
       </c>
       <c r="P27">
         <v>0</v>
@@ -3218,7 +3224,7 @@
       </c>
       <c r="K28" t="str">
         <f>$V$28</f>
-        <v>ELC</v>
+        <v>e_VN1003-500,e_VN1005-500,e_VN1008-500,e_VN1010-500,e_VN1014-500,e_VN1016-500,e_VN1019-500,e_VN1020-500,e_VN1022-500,e_VN1024-220,e_VN1130-500,e_VN1133-220,e_VN1134-220,e_VN1137-500,e_VN1138-220,e_VN1139-220,e_VN1140-500,e_VN1141-220,e_VN1141-500,e_VN1142-500,e_VN1145-220,e_VN1146-500,e_VN1147-220,e_VN1149-500,e_VN1153-220,e_VN1154-220,e_VN1157-220,e_VN1178-500,e_VN1179-220,e_VN1184-500,e_VN1187-500,e_VN1188-220,e_VN1191-500,e_VN1192-500,e_VN1196-500,e_VN1198-500,e_VN1206-220,e_VN1208-500,e_VN1209-500,e_VN1210-500,e_VN1213-220,e_VN1218-220,e_VN1219-220,e_VN1223-220,e_VN1223-500,e_VN1224-500,e_VN1226-500,e_VN1228-220,e_VN181-500,e_VN183-500,e_VN186-500,e_VN188-500,e_VN189-500,e_VN192-500,e_VN195-220,e_VN195-500,e_VN196-500,e_VN197-500,e_VN198-500,e_VN199-500,e_VN2-220,e_VN200-500,e_VN201-500,e_VN202-500,e_VN203-220,e_VN203-500,e_VN205-500,e_VN206-500,e_VN207-500,e_VN209-220,e_VN210-500,e_VN211-500,e_VN212-500,e_VN213-500,e_VN214-500,e_VN215-500,e_VN216-500,e_VN217-500,e_VN218-500,e_VN224-500,e_VN225-500,e_VN226-500,e_VN229-500,e_VN230-220,e_VN230-500,e_VN232-220,e_VN251-220,e_VN252-220,e_VN274-220,e_VN310-220,e_VN323-500,e_VN328-500,e_VN334-500,e_VN365-220,e_VN383-220,e_VN391-500,e_VN392-500,e_VN393-500,e_VN394-500,e_VN395-500,e_VN396-500,e_VN397-500,e_VN398-500,e_VN400-500,e_VN401-500,e_VN402-500,e_VN404-500,e_VN405-500,e_VN406-500,e_VN408-220,e_VN408-500,e_VN409-500,e_VN410-220,e_VN411-500,e_VN412-500,e_VN413-220,e_VN414-500,e_VN418-500,e_VN419-500,e_VN421-500,e_VN422-500,e_VN427-500,e_VN428-500,e_VN429-500,e_VN430-500,e_VN431-500,e_VN432-500,e_VN433-500,e_VN434-500,e_VN435-500,e_VN436-500,e_VN437-500,e_VN438-500,e_VN439-500,e_VN440-500,e_VN441-500,e_VN442-500,e_VN449-500,e_VN451-220,e_VN452-500,e_VN454-500,e_VN455-500,e_VN509-500,e_VN511-220,e_VN511-500,e_VN512-500,e_VN513-500,e_VN514-500,e_VN515-500,e_VN516-500,e_VN517-500,e_VN518-500,e_VN519-220,e_VN519-500,e_VN520-500,e_VN521-220,e_VN521-500,e_VN522-500,e_VN523-500,e_VN524-500,e_VN525-500,e_VN526-500,e_VN527-500,e_VN528-500,e_VN529-500,e_VN533-220,e_VN534-220,e_VN534-500,e_VN536-220,e_VN537-220,e_VN538-220,e_VN539-220,e_VN540-220,e_VN589-500,e_VN592-500,e_VN595-500,e_VN597-500,e_VN598-500,e_VN624-220,e_VN801-500,e_VN802-500,e_VN803-500,e_VN805-500,e_VN806-500,e_VN807-500,e_VN813-500,e_VN814-500,e_VN815-500,e_VN819-500,e_VN823-500,e_VN824-500,e_VN825-500,e_VN826-500,e_VN836-220,e_VN837-220,e_VN902-220,e_VN937-220,e_VN988-220,e_VN994-500,e_VN998-500,e_VN999-500,e_w1018528434-220,e_w1044469623-220,e_w1045125739-220,e_w1047280375-220,e_w1047400696-220,e_w1047400696-500,e_w1052065872-220,e_w1052125064-220,e_w1087113517-220,e_w1091686589-220,e_w1091782693-220,e_w1176845159-220,e_w1176845164-220,e_w1183902227-500,e_w1216970886-220,e_w1216970886-500,e_w1245195233-220,e_w1258175914-220,e_w1265274413-220,e_w1265274426-500,e_w1265612937-220,e_w1272088369-220,e_w1273255946-220,e_w1273527149-220,e_w1273527210-220,e_w1273948701-220,e_w1274076450-220,e_w1274076450-500,e_w1274466549-220,e_w1320784083-220,e_w1320784083-500,e_w1374565925-220,e_w1376430795-220,e_w1376430795-500,e_w241065371-220,e_w306295536-220,e_w306295536-500,e_w306295540-220,e_w307638314-220,e_w315766007-220,e_w315766015-220,e_w400645442-220,e_w400791086-220,e_w400791086-500,e_w401042494-220,e_w401532710-220,e_w468821783-220,e_w468821783-500,e_w548717060-220,e_w548717060-500,e_w548723124-220,e_w548752026-220,e_w548869165-220,e_w548869165-230,e_w548970118-220,e_w549038673-220,e_w549296358-220,e_w549380074-220,e_w549400050-220,e_w549400050-500,e_w549400051-220,e_w549577079-220,e_w549914200-220,e_w549941525-220,e_w549959350-220,e_w549959354-220,e_w630750798-220,e_w630750798-500,e_w715041211-220,e_w744217936-220,e_w762471641-220,e_w827889590-500,e_w827889600-220,e_w827889600-500,e_w967849373-220</v>
       </c>
       <c r="P28">
         <v>0</v>
@@ -3233,7 +3239,7 @@
         <v>50</v>
       </c>
       <c r="V28" s="147" t="s">
-        <v>19</v>
+        <v>393</v>
       </c>
     </row>
   </sheetData>
@@ -4710,9 +4716,8 @@
     <row r="8" spans="2:25" ht="17.649999999999999">
       <c r="B8" s="20"/>
       <c r="E8" s="26"/>
-      <c r="F8" t="str">
-        <f>C5</f>
-        <v>ELC</v>
+      <c r="F8" t="s">
+        <v>163</v>
       </c>
       <c r="G8" t="str">
         <f>E7</f>
@@ -6035,62 +6040,62 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EC20741C-AEB3-42E1-8B22-A53B1732C972}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C2FC12C8-D392-4207-9C52-F3D914A21676}">
   <dimension ref="B9:M34"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
     <row r="9" spans="2:13">
       <c r="B9" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="J9" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
     </row>
     <row r="10" spans="2:13">
       <c r="B10" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="C10" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="D10" t="s">
+        <v>167</v>
+      </c>
+      <c r="E10" t="s">
+        <v>168</v>
+      </c>
+      <c r="F10" t="s">
+        <v>169</v>
+      </c>
+      <c r="G10" t="s">
+        <v>170</v>
+      </c>
+      <c r="H10" t="s">
+        <v>171</v>
+      </c>
+      <c r="J10" t="s">
         <v>166</v>
       </c>
-      <c r="E10" t="s">
-        <v>167</v>
-      </c>
-      <c r="F10" t="s">
-        <v>168</v>
-      </c>
-      <c r="G10" t="s">
-        <v>169</v>
-      </c>
-      <c r="H10" t="s">
-        <v>170</v>
-      </c>
-      <c r="J10" t="s">
-        <v>165</v>
-      </c>
       <c r="K10" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="L10" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="M10" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
     </row>
     <row r="11" spans="2:13">
       <c r="B11" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C11" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="D11" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="E11" t="s">
         <v>10</v>
@@ -6099,16 +6104,16 @@
         <v>21</v>
       </c>
       <c r="G11" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H11" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J11" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="K11" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="L11">
         <v>8.2345024949489236</v>
@@ -6119,13 +6124,13 @@
     </row>
     <row r="12" spans="2:13">
       <c r="B12" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C12" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="D12" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="E12" t="s">
         <v>10</v>
@@ -6134,16 +6139,16 @@
         <v>21</v>
       </c>
       <c r="G12" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H12" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J12" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="K12" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="L12">
         <v>9.6220279244348106</v>
@@ -6154,13 +6159,13 @@
     </row>
     <row r="13" spans="2:13">
       <c r="B13" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C13" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="D13" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="E13" t="s">
         <v>10</v>
@@ -6169,16 +6174,16 @@
         <v>21</v>
       </c>
       <c r="G13" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H13" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J13" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="K13" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="L13">
         <v>12.989120683451539</v>
@@ -6189,13 +6194,13 @@
     </row>
     <row r="14" spans="2:13">
       <c r="B14" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C14" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="D14" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="E14" t="s">
         <v>10</v>
@@ -6204,16 +6209,16 @@
         <v>21</v>
       </c>
       <c r="G14" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H14" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J14" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="K14" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="L14">
         <v>23.367774626272176</v>
@@ -6224,13 +6229,13 @@
     </row>
     <row r="15" spans="2:13">
       <c r="B15" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C15" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="D15" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="E15" t="s">
         <v>10</v>
@@ -6239,16 +6244,16 @@
         <v>21</v>
       </c>
       <c r="G15" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H15" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J15" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="K15" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="L15">
         <v>10.064935549509592</v>
@@ -6259,13 +6264,13 @@
     </row>
     <row r="16" spans="2:13">
       <c r="B16" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C16" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="D16" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="E16" t="s">
         <v>10</v>
@@ -6274,16 +6279,16 @@
         <v>21</v>
       </c>
       <c r="G16" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H16" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J16" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="K16" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="L16">
         <v>28.968703308044521</v>
@@ -6294,13 +6299,13 @@
     </row>
     <row r="17" spans="2:13">
       <c r="B17" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C17" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="D17" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="E17" t="s">
         <v>10</v>
@@ -6309,16 +6314,16 @@
         <v>21</v>
       </c>
       <c r="G17" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H17" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J17" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="K17" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="L17">
         <v>36.409765920639195</v>
@@ -6329,13 +6334,13 @@
     </row>
     <row r="18" spans="2:13">
       <c r="B18" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C18" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="D18" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="E18" t="s">
         <v>10</v>
@@ -6344,16 +6349,16 @@
         <v>21</v>
       </c>
       <c r="G18" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H18" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J18" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="K18" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="L18">
         <v>61.629939503272361</v>
@@ -6364,13 +6369,13 @@
     </row>
     <row r="19" spans="2:13">
       <c r="B19" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C19" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="D19" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="E19" t="s">
         <v>10</v>
@@ -6379,16 +6384,16 @@
         <v>21</v>
       </c>
       <c r="G19" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H19" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J19" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="K19" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="L19">
         <v>23.184367492959971</v>
@@ -6399,13 +6404,13 @@
     </row>
     <row r="20" spans="2:13">
       <c r="B20" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C20" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="D20" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="E20" t="s">
         <v>10</v>
@@ -6414,16 +6419,16 @@
         <v>21</v>
       </c>
       <c r="G20" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H20" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J20" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="K20" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="L20">
         <v>9.4197379963727919</v>
@@ -6434,13 +6439,13 @@
     </row>
     <row r="21" spans="2:13">
       <c r="B21" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C21" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="D21" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="E21" t="s">
         <v>10</v>
@@ -6449,16 +6454,16 @@
         <v>21</v>
       </c>
       <c r="G21" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H21" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J21" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="K21" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="L21">
         <v>0.33794886068405022</v>
@@ -6469,13 +6474,13 @@
     </row>
     <row r="22" spans="2:13">
       <c r="B22" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C22" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="D22" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="E22" t="s">
         <v>10</v>
@@ -6484,16 +6489,16 @@
         <v>21</v>
       </c>
       <c r="G22" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H22" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J22" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="K22" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="L22">
         <v>15.301231471823185</v>
@@ -6504,13 +6509,13 @@
     </row>
     <row r="23" spans="2:13">
       <c r="B23" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C23" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="D23" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="E23" t="s">
         <v>10</v>
@@ -6519,16 +6524,16 @@
         <v>21</v>
       </c>
       <c r="G23" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H23" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J23" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="K23" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="L23">
         <v>1.8441823869625056</v>
@@ -6539,13 +6544,13 @@
     </row>
     <row r="24" spans="2:13">
       <c r="B24" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C24" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D24" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="E24" t="s">
         <v>10</v>
@@ -6554,16 +6559,16 @@
         <v>21</v>
       </c>
       <c r="G24" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H24" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J24" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="K24" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="L24">
         <v>8.1418373384366056</v>
@@ -6574,13 +6579,13 @@
     </row>
     <row r="25" spans="2:13">
       <c r="B25" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C25" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="D25" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="E25" t="s">
         <v>10</v>
@@ -6589,16 +6594,16 @@
         <v>21</v>
       </c>
       <c r="G25" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H25" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J25" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="K25" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="L25">
         <v>15.630231113505582</v>
@@ -6609,13 +6614,13 @@
     </row>
     <row r="26" spans="2:13">
       <c r="B26" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C26" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="D26" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="E26" t="s">
         <v>10</v>
@@ -6624,16 +6629,16 @@
         <v>21</v>
       </c>
       <c r="G26" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H26" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J26" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="K26" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="L26">
         <v>3.8834634407865751</v>
@@ -6644,13 +6649,13 @@
     </row>
     <row r="27" spans="2:13">
       <c r="B27" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C27" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="D27" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="E27" t="s">
         <v>10</v>
@@ -6659,16 +6664,16 @@
         <v>21</v>
       </c>
       <c r="G27" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H27" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J27" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="K27" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="L27">
         <v>1.3154941800590325</v>
@@ -6679,13 +6684,13 @@
     </row>
     <row r="28" spans="2:13">
       <c r="B28" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C28" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="D28" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="E28" t="s">
         <v>10</v>
@@ -6694,16 +6699,16 @@
         <v>21</v>
       </c>
       <c r="G28" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H28" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J28" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="K28" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="L28">
         <v>0.96790070270628858</v>
@@ -6714,13 +6719,13 @@
     </row>
     <row r="29" spans="2:13">
       <c r="B29" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C29" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="D29" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="E29" t="s">
         <v>10</v>
@@ -6729,16 +6734,16 @@
         <v>21</v>
       </c>
       <c r="G29" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H29" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J29" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="K29" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="L29">
         <v>24.150858853338818</v>
@@ -6749,13 +6754,13 @@
     </row>
     <row r="30" spans="2:13">
       <c r="B30" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C30" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="D30" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="E30" t="s">
         <v>10</v>
@@ -6764,16 +6769,16 @@
         <v>21</v>
       </c>
       <c r="G30" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H30" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J30" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="K30" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="L30">
         <v>8.2395742020356355</v>
@@ -6784,13 +6789,13 @@
     </row>
     <row r="31" spans="2:13">
       <c r="B31" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C31" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="D31" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="E31" t="s">
         <v>10</v>
@@ -6799,16 +6804,16 @@
         <v>21</v>
       </c>
       <c r="G31" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H31" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J31" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="K31" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="L31">
         <v>1.1031656597894786</v>
@@ -6819,13 +6824,13 @@
     </row>
     <row r="32" spans="2:13">
       <c r="B32" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C32" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="D32" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="E32" t="s">
         <v>10</v>
@@ -6834,16 +6839,16 @@
         <v>21</v>
       </c>
       <c r="G32" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H32" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J32" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="K32" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="L32">
         <v>4.3671750196561172</v>
@@ -6854,13 +6859,13 @@
     </row>
     <row r="33" spans="2:13">
       <c r="B33" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C33" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="D33" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="E33" t="s">
         <v>10</v>
@@ -6869,16 +6874,16 @@
         <v>21</v>
       </c>
       <c r="G33" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H33" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J33" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="K33" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="L33">
         <v>0.85339138388924274</v>
@@ -6889,13 +6894,13 @@
     </row>
     <row r="34" spans="2:13">
       <c r="B34" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C34" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="D34" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="E34" t="s">
         <v>10</v>
@@ -6904,16 +6909,16 @@
         <v>21</v>
       </c>
       <c r="G34" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H34" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J34" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="K34" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="L34">
         <v>4.3661509546498927</v>
@@ -6928,101 +6933,101 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{21C08DBD-6CFC-4BE5-9C22-4295557F1C98}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA8FD518-8FA8-440B-93A7-DE2F4E0BB7ED}">
   <dimension ref="B9:Z32"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
     <row r="9" spans="2:26">
       <c r="B9" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="J9" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="O9" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="W9" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
     </row>
     <row r="10" spans="2:26">
       <c r="B10" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="C10" t="s">
+        <v>166</v>
+      </c>
+      <c r="D10" t="s">
+        <v>167</v>
+      </c>
+      <c r="E10" t="s">
+        <v>168</v>
+      </c>
+      <c r="F10" t="s">
+        <v>169</v>
+      </c>
+      <c r="G10" t="s">
+        <v>170</v>
+      </c>
+      <c r="H10" t="s">
+        <v>171</v>
+      </c>
+      <c r="J10" t="s">
+        <v>166</v>
+      </c>
+      <c r="K10" t="s">
+        <v>224</v>
+      </c>
+      <c r="L10" t="s">
+        <v>225</v>
+      </c>
+      <c r="M10" t="s">
+        <v>226</v>
+      </c>
+      <c r="O10" t="s">
         <v>165</v>
       </c>
-      <c r="D10" t="s">
+      <c r="P10" t="s">
         <v>166</v>
       </c>
-      <c r="E10" t="s">
+      <c r="Q10" t="s">
         <v>167</v>
       </c>
-      <c r="F10" t="s">
+      <c r="R10" t="s">
         <v>168</v>
       </c>
-      <c r="G10" t="s">
+      <c r="S10" t="s">
         <v>169</v>
       </c>
-      <c r="H10" t="s">
+      <c r="T10" t="s">
         <v>170</v>
       </c>
-      <c r="J10" t="s">
-        <v>165</v>
-      </c>
-      <c r="K10" t="s">
-        <v>223</v>
-      </c>
-      <c r="L10" t="s">
+      <c r="U10" t="s">
+        <v>171</v>
+      </c>
+      <c r="W10" t="s">
+        <v>166</v>
+      </c>
+      <c r="X10" t="s">
         <v>224</v>
       </c>
-      <c r="M10" t="s">
+      <c r="Y10" t="s">
         <v>225</v>
       </c>
-      <c r="O10" t="s">
-        <v>164</v>
-      </c>
-      <c r="P10" t="s">
-        <v>165</v>
-      </c>
-      <c r="Q10" t="s">
-        <v>166</v>
-      </c>
-      <c r="R10" t="s">
-        <v>167</v>
-      </c>
-      <c r="S10" t="s">
-        <v>168</v>
-      </c>
-      <c r="T10" t="s">
-        <v>169</v>
-      </c>
-      <c r="U10" t="s">
-        <v>170</v>
-      </c>
-      <c r="W10" t="s">
-        <v>165</v>
-      </c>
-      <c r="X10" t="s">
-        <v>223</v>
-      </c>
-      <c r="Y10" t="s">
-        <v>224</v>
-      </c>
       <c r="Z10" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
     </row>
     <row r="11" spans="2:26">
       <c r="B11" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C11" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="D11" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="E11" t="s">
         <v>10</v>
@@ -7031,16 +7036,16 @@
         <v>21</v>
       </c>
       <c r="G11" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H11" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J11" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="K11" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="L11">
         <v>9.9561879268440521</v>
@@ -7049,13 +7054,13 @@
         <v>0.20471165282517209</v>
       </c>
       <c r="O11" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="P11" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="Q11" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="R11" t="s">
         <v>10</v>
@@ -7064,16 +7069,16 @@
         <v>21</v>
       </c>
       <c r="T11" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="U11" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="W11" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="X11" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="Y11">
         <v>5.7030000000000003</v>
@@ -7084,13 +7089,13 @@
     </row>
     <row r="12" spans="2:26">
       <c r="B12" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C12" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="D12" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="E12" t="s">
         <v>10</v>
@@ -7099,16 +7104,16 @@
         <v>21</v>
       </c>
       <c r="G12" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H12" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J12" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="K12" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="L12">
         <v>15.610469208056319</v>
@@ -7117,13 +7122,13 @@
         <v>0.1506732372188746</v>
       </c>
       <c r="O12" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="P12" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="Q12" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="R12" t="s">
         <v>10</v>
@@ -7132,16 +7137,16 @@
         <v>21</v>
       </c>
       <c r="T12" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="U12" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="W12" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="X12" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="Y12">
         <v>3.2370000000000001</v>
@@ -7152,13 +7157,13 @@
     </row>
     <row r="13" spans="2:26">
       <c r="B13" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C13" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="D13" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="E13" t="s">
         <v>10</v>
@@ -7167,16 +7172,16 @@
         <v>21</v>
       </c>
       <c r="G13" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H13" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J13" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="K13" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="L13">
         <v>38.93604588989777</v>
@@ -7185,13 +7190,13 @@
         <v>0.1218221396795726</v>
       </c>
       <c r="O13" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="P13" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="Q13" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="R13" t="s">
         <v>10</v>
@@ -7200,16 +7205,16 @@
         <v>21</v>
       </c>
       <c r="T13" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="U13" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="W13" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="X13" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="Y13">
         <v>0.73950000000000005</v>
@@ -7220,13 +7225,13 @@
     </row>
     <row r="14" spans="2:26">
       <c r="B14" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C14" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="D14" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="E14" t="s">
         <v>10</v>
@@ -7235,16 +7240,16 @@
         <v>21</v>
       </c>
       <c r="G14" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H14" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J14" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="K14" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="L14">
         <v>3.4061833906252343</v>
@@ -7253,13 +7258,13 @@
         <v>0.1484206750914133</v>
       </c>
       <c r="O14" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="P14" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="Q14" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="R14" t="s">
         <v>10</v>
@@ -7268,16 +7273,16 @@
         <v>21</v>
       </c>
       <c r="T14" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="U14" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="W14" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="X14" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="Y14">
         <v>17.418749999999999</v>
@@ -7288,13 +7293,13 @@
     </row>
     <row r="15" spans="2:26">
       <c r="B15" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C15" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="D15" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="E15" t="s">
         <v>10</v>
@@ -7303,16 +7308,16 @@
         <v>21</v>
       </c>
       <c r="G15" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H15" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J15" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="K15" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="L15">
         <v>10.05531955531686</v>
@@ -7321,13 +7326,13 @@
         <v>0.2184912647230102</v>
       </c>
       <c r="O15" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="P15" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="Q15" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="R15" t="s">
         <v>10</v>
@@ -7336,16 +7341,16 @@
         <v>21</v>
       </c>
       <c r="T15" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="U15" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="W15" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="X15" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="Y15">
         <v>75.501750000000001</v>
@@ -7356,13 +7361,13 @@
     </row>
     <row r="16" spans="2:26">
       <c r="B16" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C16" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="D16" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="E16" t="s">
         <v>10</v>
@@ -7371,16 +7376,16 @@
         <v>21</v>
       </c>
       <c r="G16" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H16" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J16" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="K16" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="L16">
         <v>11.000319473014851</v>
@@ -7389,13 +7394,13 @@
         <v>0.1122659335993704</v>
       </c>
       <c r="O16" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="P16" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="Q16" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="R16" t="s">
         <v>10</v>
@@ -7404,16 +7409,16 @@
         <v>21</v>
       </c>
       <c r="T16" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="U16" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="W16" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="X16" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="Y16">
         <v>26.099250000000001</v>
@@ -7424,13 +7429,13 @@
     </row>
     <row r="17" spans="2:26">
       <c r="B17" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C17" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="D17" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="E17" t="s">
         <v>10</v>
@@ -7439,16 +7444,16 @@
         <v>21</v>
       </c>
       <c r="G17" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H17" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J17" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="K17" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="L17">
         <v>1.9758785540112649</v>
@@ -7457,13 +7462,13 @@
         <v>0.196320507772859</v>
       </c>
       <c r="O17" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="P17" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="Q17" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="R17" t="s">
         <v>10</v>
@@ -7472,16 +7477,16 @@
         <v>21</v>
       </c>
       <c r="T17" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="U17" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="W17" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="X17" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="Y17">
         <v>6.7657499999999997</v>
@@ -7492,13 +7497,13 @@
     </row>
     <row r="18" spans="2:26">
       <c r="B18" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C18" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="D18" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="E18" t="s">
         <v>10</v>
@@ -7507,16 +7512,16 @@
         <v>21</v>
       </c>
       <c r="G18" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H18" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J18" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="K18" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="L18">
         <v>10.302711276720984</v>
@@ -7525,13 +7530,13 @@
         <v>0.1557497332814953</v>
       </c>
       <c r="O18" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="P18" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="Q18" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="R18" t="s">
         <v>10</v>
@@ -7540,16 +7545,16 @@
         <v>21</v>
       </c>
       <c r="T18" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="U18" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="W18" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="X18" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="Y18">
         <v>18.204750000000001</v>
@@ -7560,13 +7565,13 @@
     </row>
     <row r="19" spans="2:26">
       <c r="B19" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C19" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="D19" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="E19" t="s">
         <v>10</v>
@@ -7575,16 +7580,16 @@
         <v>21</v>
       </c>
       <c r="G19" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H19" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J19" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="K19" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="L19">
         <v>21.084725957939643</v>
@@ -7593,13 +7598,13 @@
         <v>0.13822135063727131</v>
       </c>
       <c r="O19" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="P19" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="Q19" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="R19" t="s">
         <v>10</v>
@@ -7608,16 +7613,16 @@
         <v>21</v>
       </c>
       <c r="T19" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="U19" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="W19" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="X19" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="Y19">
         <v>53.964750000000002</v>
@@ -7628,13 +7633,13 @@
     </row>
     <row r="20" spans="2:26">
       <c r="B20" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C20" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="D20" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="E20" t="s">
         <v>10</v>
@@ -7643,16 +7648,16 @@
         <v>21</v>
       </c>
       <c r="G20" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H20" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J20" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="K20" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="L20">
         <v>7.8234985450080243</v>
@@ -7661,13 +7666,13 @@
         <v>0.13991196104030729</v>
       </c>
       <c r="O20" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="P20" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="Q20" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="R20" t="s">
         <v>10</v>
@@ -7676,16 +7681,16 @@
         <v>21</v>
       </c>
       <c r="T20" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="U20" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="W20" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="X20" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="Y20">
         <v>32.474249999999998</v>
@@ -7696,13 +7701,13 @@
     </row>
     <row r="21" spans="2:26">
       <c r="B21" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C21" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="D21" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="E21" t="s">
         <v>10</v>
@@ -7711,16 +7716,16 @@
         <v>21</v>
       </c>
       <c r="G21" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H21" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J21" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="K21" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="L21">
         <v>35.48135454794123</v>
@@ -7729,13 +7734,13 @@
         <v>0.16865809324234321</v>
       </c>
       <c r="O21" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="P21" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="Q21" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="R21" t="s">
         <v>10</v>
@@ -7744,16 +7749,16 @@
         <v>21</v>
       </c>
       <c r="T21" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="U21" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="W21" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="X21" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="Y21">
         <v>24.771750000000001</v>
@@ -7764,13 +7769,13 @@
     </row>
     <row r="22" spans="2:26">
       <c r="B22" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C22" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="D22" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="E22" t="s">
         <v>10</v>
@@ -7779,16 +7784,16 @@
         <v>21</v>
       </c>
       <c r="G22" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H22" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J22" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="K22" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="L22">
         <v>31.11916467188631</v>
@@ -7797,13 +7802,13 @@
         <v>0.18949756193894909</v>
       </c>
       <c r="O22" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="P22" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="Q22" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="R22" t="s">
         <v>10</v>
@@ -7812,16 +7817,16 @@
         <v>21</v>
       </c>
       <c r="T22" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="U22" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="W22" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="X22" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="Y22">
         <v>34.518000000000001</v>
@@ -7832,13 +7837,13 @@
     </row>
     <row r="23" spans="2:26">
       <c r="B23" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C23" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="D23" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="E23" t="s">
         <v>10</v>
@@ -7847,16 +7852,16 @@
         <v>21</v>
       </c>
       <c r="G23" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H23" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J23" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="K23" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="L23">
         <v>4.5001608244833662</v>
@@ -7865,13 +7870,13 @@
         <v>0.12594720676955351</v>
       </c>
       <c r="O23" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="P23" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="Q23" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="R23" t="s">
         <v>10</v>
@@ -7880,16 +7885,16 @@
         <v>21</v>
       </c>
       <c r="T23" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="U23" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="W23" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="X23" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="Y23">
         <v>13.3995</v>
@@ -7900,13 +7905,13 @@
     </row>
     <row r="24" spans="2:26">
       <c r="B24" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C24" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="D24" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="E24" t="s">
         <v>10</v>
@@ -7915,16 +7920,16 @@
         <v>21</v>
       </c>
       <c r="G24" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H24" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J24" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="K24" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="L24">
         <v>9.5500952124569967</v>
@@ -7933,13 +7938,13 @@
         <v>0.19448607563648629</v>
       </c>
       <c r="O24" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="P24" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="Q24" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="R24" t="s">
         <v>10</v>
@@ -7948,16 +7953,16 @@
         <v>21</v>
       </c>
       <c r="T24" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="U24" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="W24" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="X24" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="Y24">
         <v>38.413499999999999</v>
@@ -7968,13 +7973,13 @@
     </row>
     <row r="25" spans="2:26">
       <c r="B25" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C25" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="D25" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="E25" t="s">
         <v>10</v>
@@ -7983,16 +7988,16 @@
         <v>21</v>
       </c>
       <c r="G25" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H25" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J25" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="K25" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="L25">
         <v>5.3426370365388722</v>
@@ -8001,13 +8006,13 @@
         <v>0.15993664446002681</v>
       </c>
       <c r="O25" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="P25" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="Q25" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="R25" t="s">
         <v>10</v>
@@ -8016,16 +8021,16 @@
         <v>21</v>
       </c>
       <c r="T25" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="U25" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="W25" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="X25" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="Y25">
         <v>15.254250000000001</v>
@@ -8036,13 +8041,13 @@
     </row>
     <row r="26" spans="2:26">
       <c r="B26" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C26" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="D26" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="E26" t="s">
         <v>10</v>
@@ -8051,16 +8056,16 @@
         <v>21</v>
       </c>
       <c r="G26" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H26" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J26" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="K26" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="L26">
         <v>1.0928295776667281</v>
@@ -8069,13 +8074,13 @@
         <v>0.15944636785409541</v>
       </c>
       <c r="O26" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="P26" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="Q26" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="R26" t="s">
         <v>10</v>
@@ -8084,16 +8089,16 @@
         <v>21</v>
       </c>
       <c r="T26" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="U26" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="W26" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="X26" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="Y26">
         <v>16.820250000000001</v>
@@ -8104,13 +8109,13 @@
     </row>
     <row r="27" spans="2:26">
       <c r="B27" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C27" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="D27" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="E27" t="s">
         <v>10</v>
@@ -8119,16 +8124,16 @@
         <v>21</v>
       </c>
       <c r="G27" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H27" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J27" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="K27" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="L27">
         <v>0.94607061901700107</v>
@@ -8137,13 +8142,13 @@
         <v>0.18581643202413151</v>
       </c>
       <c r="O27" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="P27" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="Q27" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="R27" t="s">
         <v>10</v>
@@ -8152,16 +8157,16 @@
         <v>21</v>
       </c>
       <c r="T27" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="U27" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="W27" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="X27" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="Y27">
         <v>32.364750000000001</v>
@@ -8172,13 +8177,13 @@
     </row>
     <row r="28" spans="2:26">
       <c r="O28" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="P28" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="Q28" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="R28" t="s">
         <v>10</v>
@@ -8187,16 +8192,16 @@
         <v>21</v>
       </c>
       <c r="T28" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="U28" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="W28" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="X28" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="Y28">
         <v>20.224499999999999</v>
@@ -8207,13 +8212,13 @@
     </row>
     <row r="29" spans="2:26">
       <c r="O29" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="P29" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="Q29" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="R29" t="s">
         <v>10</v>
@@ -8222,16 +8227,16 @@
         <v>21</v>
       </c>
       <c r="T29" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="U29" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="W29" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="X29" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="Y29">
         <v>13.347</v>
@@ -8242,13 +8247,13 @@
     </row>
     <row r="30" spans="2:26">
       <c r="O30" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="P30" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="Q30" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="R30" t="s">
         <v>10</v>
@@ -8257,16 +8262,16 @@
         <v>21</v>
       </c>
       <c r="T30" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="U30" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="W30" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="X30" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="Y30">
         <v>3.7177500000000001</v>
@@ -8277,13 +8282,13 @@
     </row>
     <row r="31" spans="2:26">
       <c r="O31" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="P31" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="Q31" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="R31" t="s">
         <v>10</v>
@@ -8292,16 +8297,16 @@
         <v>21</v>
       </c>
       <c r="T31" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="U31" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="W31" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="X31" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="Y31">
         <v>9.6434999999999995</v>
@@ -8312,13 +8317,13 @@
     </row>
     <row r="32" spans="2:26">
       <c r="O32" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="P32" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="Q32" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="R32" t="s">
         <v>10</v>
@@ -8327,16 +8332,16 @@
         <v>21</v>
       </c>
       <c r="T32" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="U32" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="W32" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="X32" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="Y32">
         <v>38.509500000000003</v>
@@ -8351,27 +8356,27 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4F18ABC8-0759-4F51-AC5E-310364C2142E}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5065A376-F302-40DE-88C4-7F9FCAA092A8}">
   <dimension ref="B9:P73"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
     <row r="9" spans="2:16">
       <c r="B9" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="J9" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
     </row>
     <row r="10" spans="2:16">
       <c r="B10" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="C10" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="D10" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="E10">
         <v>2023</v>
@@ -8386,30 +8391,30 @@
         <v>54</v>
       </c>
       <c r="J10" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="K10" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="L10" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="M10" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="N10" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="O10" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="P10" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
     </row>
     <row r="11" spans="2:16">
       <c r="B11" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="C11" t="s">
         <v>31</v>
@@ -8430,10 +8435,10 @@
         <v>146</v>
       </c>
       <c r="J11" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="K11" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="M11" t="s">
         <v>10</v>
@@ -8442,15 +8447,15 @@
         <v>21</v>
       </c>
       <c r="O11" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="P11" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
     </row>
     <row r="12" spans="2:16">
       <c r="B12" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="C12" t="s">
         <v>31</v>
@@ -8468,13 +8473,13 @@
         <v>0.60000000000000009</v>
       </c>
       <c r="H12" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="J12" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="K12" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="M12" t="s">
         <v>10</v>
@@ -8483,15 +8488,15 @@
         <v>21</v>
       </c>
       <c r="O12" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="P12" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
     </row>
     <row r="13" spans="2:16">
       <c r="B13" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="C13" t="s">
         <v>31</v>
@@ -8509,13 +8514,13 @@
         <v>4200</v>
       </c>
       <c r="H13" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="J13" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="K13" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="M13" t="s">
         <v>10</v>
@@ -8524,15 +8529,15 @@
         <v>21</v>
       </c>
       <c r="O13" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="P13" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
     </row>
     <row r="14" spans="2:16">
       <c r="B14" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="C14" t="s">
         <v>31</v>
@@ -8550,13 +8555,13 @@
         <v>145</v>
       </c>
       <c r="H14" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="J14" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="K14" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="M14" t="s">
         <v>10</v>
@@ -8565,15 +8570,15 @@
         <v>21</v>
       </c>
       <c r="O14" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="P14" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
     </row>
     <row r="15" spans="2:16">
       <c r="B15" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="C15" t="s">
         <v>31</v>
@@ -8591,13 +8596,13 @@
         <v>3</v>
       </c>
       <c r="H15" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="J15" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="K15" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="M15" t="s">
         <v>10</v>
@@ -8606,15 +8611,15 @@
         <v>21</v>
       </c>
       <c r="O15" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="P15" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
     </row>
     <row r="16" spans="2:16">
       <c r="B16" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="C16" t="s">
         <v>31</v>
@@ -8635,10 +8640,10 @@
         <v>146</v>
       </c>
       <c r="J16" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="K16" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="M16" t="s">
         <v>10</v>
@@ -8647,15 +8652,15 @@
         <v>21</v>
       </c>
       <c r="O16" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="P16" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
     </row>
     <row r="17" spans="2:16">
       <c r="B17" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="C17" t="s">
         <v>31</v>
@@ -8673,13 +8678,13 @@
         <v>0.60000000000000009</v>
       </c>
       <c r="H17" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="J17" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="K17" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="M17" t="s">
         <v>10</v>
@@ -8688,15 +8693,15 @@
         <v>21</v>
       </c>
       <c r="O17" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="P17" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
     </row>
     <row r="18" spans="2:16">
       <c r="B18" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="C18" t="s">
         <v>31</v>
@@ -8714,13 +8719,13 @@
         <v>2050</v>
       </c>
       <c r="H18" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="J18" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="K18" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="M18" t="s">
         <v>10</v>
@@ -8729,15 +8734,15 @@
         <v>21</v>
       </c>
       <c r="O18" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="P18" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
     </row>
     <row r="19" spans="2:16">
       <c r="B19" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="C19" t="s">
         <v>31</v>
@@ -8755,13 +8760,13 @@
         <v>70</v>
       </c>
       <c r="H19" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="J19" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="K19" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="M19" t="s">
         <v>10</v>
@@ -8770,15 +8775,15 @@
         <v>21</v>
       </c>
       <c r="O19" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="P19" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
     </row>
     <row r="20" spans="2:16">
       <c r="B20" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="C20" t="s">
         <v>31</v>
@@ -8796,13 +8801,13 @@
         <v>3</v>
       </c>
       <c r="H20" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="J20" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="K20" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="M20" t="s">
         <v>10</v>
@@ -8811,15 +8816,15 @@
         <v>21</v>
       </c>
       <c r="O20" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="P20" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
     </row>
     <row r="21" spans="2:16">
       <c r="B21" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="C21" t="s">
         <v>33</v>
@@ -8840,10 +8845,10 @@
         <v>146</v>
       </c>
       <c r="J21" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="K21" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="M21" t="s">
         <v>10</v>
@@ -8852,15 +8857,15 @@
         <v>21</v>
       </c>
       <c r="O21" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="P21" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
     </row>
     <row r="22" spans="2:16">
       <c r="B22" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="C22" t="s">
         <v>33</v>
@@ -8878,13 +8883,13 @@
         <v>700</v>
       </c>
       <c r="H22" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="J22" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="K22" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="M22" t="s">
         <v>10</v>
@@ -8893,15 +8898,15 @@
         <v>21</v>
       </c>
       <c r="O22" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="P22" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
     </row>
     <row r="23" spans="2:16">
       <c r="B23" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="C23" t="s">
         <v>33</v>
@@ -8919,13 +8924,13 @@
         <v>25</v>
       </c>
       <c r="H23" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="J23" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="K23" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="M23" t="s">
         <v>10</v>
@@ -8934,15 +8939,15 @@
         <v>21</v>
       </c>
       <c r="O23" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="P23" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
     </row>
     <row r="24" spans="2:16">
       <c r="B24" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="C24" t="s">
         <v>33</v>
@@ -8963,10 +8968,10 @@
         <v>146</v>
       </c>
       <c r="J24" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="K24" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="M24" t="s">
         <v>10</v>
@@ -8975,15 +8980,15 @@
         <v>21</v>
       </c>
       <c r="O24" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="P24" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
     </row>
     <row r="25" spans="2:16">
       <c r="B25" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="C25" t="s">
         <v>33</v>
@@ -9001,13 +9006,13 @@
         <v>1750</v>
       </c>
       <c r="H25" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="J25" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="K25" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="M25" t="s">
         <v>10</v>
@@ -9016,15 +9021,15 @@
         <v>21</v>
       </c>
       <c r="O25" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="P25" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
     </row>
     <row r="26" spans="2:16">
       <c r="B26" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="C26" t="s">
         <v>33</v>
@@ -9042,13 +9047,13 @@
         <v>60</v>
       </c>
       <c r="H26" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="J26" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="K26" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="M26" t="s">
         <v>10</v>
@@ -9057,15 +9062,15 @@
         <v>21</v>
       </c>
       <c r="O26" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="P26" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
     </row>
     <row r="27" spans="2:16">
       <c r="B27" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="C27" t="s">
         <v>32</v>
@@ -9086,10 +9091,10 @@
         <v>146</v>
       </c>
       <c r="J27" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="K27" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="M27" t="s">
         <v>10</v>
@@ -9098,15 +9103,15 @@
         <v>21</v>
       </c>
       <c r="O27" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="P27" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
     </row>
     <row r="28" spans="2:16">
       <c r="B28" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="C28" t="s">
         <v>32</v>
@@ -9124,12 +9129,12 @@
         <v>3000</v>
       </c>
       <c r="H28" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
     </row>
     <row r="29" spans="2:16">
       <c r="B29" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="C29" t="s">
         <v>32</v>
@@ -9147,12 +9152,12 @@
         <v>120</v>
       </c>
       <c r="H29" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
     </row>
     <row r="30" spans="2:16">
       <c r="B30" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="C30" t="s">
         <v>33</v>
@@ -9175,7 +9180,7 @@
     </row>
     <row r="31" spans="2:16">
       <c r="B31" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="C31" t="s">
         <v>33</v>
@@ -9193,12 +9198,12 @@
         <v>400</v>
       </c>
       <c r="H31" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
     </row>
     <row r="32" spans="2:16">
       <c r="B32" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="C32" t="s">
         <v>33</v>
@@ -9216,12 +9221,12 @@
         <v>20</v>
       </c>
       <c r="H32" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
     </row>
     <row r="33" spans="2:8">
       <c r="B33" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="C33" t="s">
         <v>28</v>
@@ -9244,7 +9249,7 @@
     </row>
     <row r="34" spans="2:8">
       <c r="B34" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="C34" t="s">
         <v>28</v>
@@ -9262,12 +9267,12 @@
         <v>0.4</v>
       </c>
       <c r="H34" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
     </row>
     <row r="35" spans="2:8">
       <c r="B35" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="C35" t="s">
         <v>28</v>
@@ -9285,12 +9290,12 @@
         <v>2000</v>
       </c>
       <c r="H35" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
     </row>
     <row r="36" spans="2:8">
       <c r="B36" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="C36" t="s">
         <v>28</v>
@@ -9308,12 +9313,12 @@
         <v>50</v>
       </c>
       <c r="H36" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
     </row>
     <row r="37" spans="2:8">
       <c r="B37" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="C37" t="s">
         <v>28</v>
@@ -9331,12 +9336,12 @@
         <v>4</v>
       </c>
       <c r="H37" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
     </row>
     <row r="38" spans="2:8">
       <c r="B38" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="C38" t="s">
         <v>33</v>
@@ -9359,7 +9364,7 @@
     </row>
     <row r="39" spans="2:8">
       <c r="B39" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="C39" t="s">
         <v>33</v>
@@ -9377,12 +9382,12 @@
         <v>1500</v>
       </c>
       <c r="H39" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
     </row>
     <row r="40" spans="2:8">
       <c r="B40" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="C40" t="s">
         <v>33</v>
@@ -9400,12 +9405,12 @@
         <v>70</v>
       </c>
       <c r="H40" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
     </row>
     <row r="41" spans="2:8">
       <c r="B41" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="C41" t="s">
         <v>32</v>
@@ -9428,7 +9433,7 @@
     </row>
     <row r="42" spans="2:8">
       <c r="B42" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="C42" t="s">
         <v>32</v>
@@ -9446,12 +9451,12 @@
         <v>3550</v>
       </c>
       <c r="H42" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
     </row>
     <row r="43" spans="2:8">
       <c r="B43" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="C43" t="s">
         <v>32</v>
@@ -9469,12 +9474,12 @@
         <v>170</v>
       </c>
       <c r="H43" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
     </row>
     <row r="44" spans="2:8">
       <c r="B44" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="C44" t="s">
         <v>36</v>
@@ -9497,7 +9502,7 @@
     </row>
     <row r="45" spans="2:8">
       <c r="B45" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="C45" t="s">
         <v>36</v>
@@ -9515,12 +9520,12 @@
         <v>2800</v>
       </c>
       <c r="H45" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
     </row>
     <row r="46" spans="2:8">
       <c r="B46" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="C46" t="s">
         <v>36</v>
@@ -9538,12 +9543,12 @@
         <v>140</v>
       </c>
       <c r="H46" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
     </row>
     <row r="47" spans="2:8">
       <c r="B47" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="C47" t="s">
         <v>32</v>
@@ -9566,7 +9571,7 @@
     </row>
     <row r="48" spans="2:8">
       <c r="B48" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="C48" t="s">
         <v>32</v>
@@ -9584,12 +9589,12 @@
         <v>3650</v>
       </c>
       <c r="H48" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
     </row>
     <row r="49" spans="2:8">
       <c r="B49" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="C49" t="s">
         <v>32</v>
@@ -9607,12 +9612,12 @@
         <v>145</v>
       </c>
       <c r="H49" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
     </row>
     <row r="50" spans="2:8">
       <c r="B50" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="C50" t="s">
         <v>27</v>
@@ -9635,7 +9640,7 @@
     </row>
     <row r="51" spans="2:8">
       <c r="B51" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="C51" t="s">
         <v>27</v>
@@ -9653,12 +9658,12 @@
         <v>0.22</v>
       </c>
       <c r="H51" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
     </row>
     <row r="52" spans="2:8">
       <c r="B52" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="C52" t="s">
         <v>27</v>
@@ -9676,12 +9681,12 @@
         <v>300</v>
       </c>
       <c r="H52" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
     </row>
     <row r="53" spans="2:8">
       <c r="B53" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="C53" t="s">
         <v>27</v>
@@ -9699,12 +9704,12 @@
         <v>10</v>
       </c>
       <c r="H53" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
     </row>
     <row r="54" spans="2:8">
       <c r="B54" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="C54" t="s">
         <v>27</v>
@@ -9722,12 +9727,12 @@
         <v>1.5</v>
       </c>
       <c r="H54" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
     </row>
     <row r="55" spans="2:8">
       <c r="B55" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="C55" t="s">
         <v>32</v>
@@ -9750,7 +9755,7 @@
     </row>
     <row r="56" spans="2:8">
       <c r="B56" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="C56" t="s">
         <v>32</v>
@@ -9768,12 +9773,12 @@
         <v>1000</v>
       </c>
       <c r="H56" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
     </row>
     <row r="57" spans="2:8">
       <c r="B57" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="C57" t="s">
         <v>32</v>
@@ -9791,12 +9796,12 @@
         <v>35</v>
       </c>
       <c r="H57" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
     </row>
     <row r="58" spans="2:8">
       <c r="B58" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="C58" t="s">
         <v>32</v>
@@ -9819,7 +9824,7 @@
     </row>
     <row r="59" spans="2:8">
       <c r="B59" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="C59" t="s">
         <v>32</v>
@@ -9837,12 +9842,12 @@
         <v>1200</v>
       </c>
       <c r="H59" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
     </row>
     <row r="60" spans="2:8">
       <c r="B60" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="C60" t="s">
         <v>32</v>
@@ -9860,12 +9865,12 @@
         <v>50</v>
       </c>
       <c r="H60" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
     </row>
     <row r="61" spans="2:8">
       <c r="B61" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="C61" t="s">
         <v>32</v>
@@ -9888,7 +9893,7 @@
     </row>
     <row r="62" spans="2:8">
       <c r="B62" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="C62" t="s">
         <v>32</v>
@@ -9906,12 +9911,12 @@
         <v>1400</v>
       </c>
       <c r="H62" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
     </row>
     <row r="63" spans="2:8">
       <c r="B63" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="C63" t="s">
         <v>32</v>
@@ -9929,15 +9934,15 @@
         <v>55</v>
       </c>
       <c r="H63" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
     </row>
     <row r="64" spans="2:8">
       <c r="B64" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="C64" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="D64" t="s">
         <v>19</v>
@@ -9957,10 +9962,10 @@
     </row>
     <row r="65" spans="2:8">
       <c r="B65" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="C65" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="D65" t="s">
         <v>19</v>
@@ -9975,15 +9980,15 @@
         <v>0.39</v>
       </c>
       <c r="H65" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
     </row>
     <row r="66" spans="2:8">
       <c r="B66" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="C66" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="D66" t="s">
         <v>19</v>
@@ -9998,15 +10003,15 @@
         <v>1360</v>
       </c>
       <c r="H66" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
     </row>
     <row r="67" spans="2:8">
       <c r="B67" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="C67" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="D67" t="s">
         <v>19</v>
@@ -10021,15 +10026,15 @@
         <v>40</v>
       </c>
       <c r="H67" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
     </row>
     <row r="68" spans="2:8">
       <c r="B68" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="C68" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="D68" t="s">
         <v>19</v>
@@ -10044,15 +10049,15 @@
         <v>3</v>
       </c>
       <c r="H68" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
     </row>
     <row r="69" spans="2:8">
       <c r="B69" t="s">
+        <v>390</v>
+      </c>
+      <c r="C69" t="s">
         <v>389</v>
-      </c>
-      <c r="C69" t="s">
-        <v>388</v>
       </c>
       <c r="D69" t="s">
         <v>19</v>
@@ -10072,10 +10077,10 @@
     </row>
     <row r="70" spans="2:8">
       <c r="B70" t="s">
+        <v>390</v>
+      </c>
+      <c r="C70" t="s">
         <v>389</v>
-      </c>
-      <c r="C70" t="s">
-        <v>388</v>
       </c>
       <c r="D70" t="s">
         <v>19</v>
@@ -10090,15 +10095,15 @@
         <v>0.3</v>
       </c>
       <c r="H70" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
     </row>
     <row r="71" spans="2:8">
       <c r="B71" t="s">
+        <v>390</v>
+      </c>
+      <c r="C71" t="s">
         <v>389</v>
-      </c>
-      <c r="C71" t="s">
-        <v>388</v>
       </c>
       <c r="D71" t="s">
         <v>19</v>
@@ -10113,15 +10118,15 @@
         <v>1090</v>
       </c>
       <c r="H71" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
     </row>
     <row r="72" spans="2:8">
       <c r="B72" t="s">
+        <v>390</v>
+      </c>
+      <c r="C72" t="s">
         <v>389</v>
-      </c>
-      <c r="C72" t="s">
-        <v>388</v>
       </c>
       <c r="D72" t="s">
         <v>19</v>
@@ -10136,15 +10141,15 @@
         <v>28</v>
       </c>
       <c r="H72" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
     </row>
     <row r="73" spans="2:8">
       <c r="B73" t="s">
+        <v>390</v>
+      </c>
+      <c r="C73" t="s">
         <v>389</v>
-      </c>
-      <c r="C73" t="s">
-        <v>388</v>
       </c>
       <c r="D73" t="s">
         <v>19</v>
@@ -10159,7 +10164,7 @@
         <v>1.5</v>
       </c>
       <c r="H73" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
     </row>
   </sheetData>

</xml_diff>